<commit_message>
excel recovery file update
</commit_message>
<xml_diff>
--- a/hw/SD-ZMB/bom/ZMB_bom-trbl.xlsx
+++ b/hw/SD-ZMB/bom/ZMB_bom-trbl.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aesil\proj\sd-zmb\hw\SD-ZMB\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BA1C5270-8555-4D2D-9971-789277E06C53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E8A554E-769E-4FC2-BD22-C0FCF30D5543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="277" windowWidth="21270" windowHeight="13403" xr2:uid="{F2BCCDDA-634B-4080-8A00-CCE749818308}"/>
+    <workbookView xWindow="1770" yWindow="997" windowWidth="21270" windowHeight="13403" xr2:uid="{F2BCCDDA-634B-4080-8A00-CCE749818308}"/>
   </bookViews>
   <sheets>
     <sheet name="ZMB_bom-trbl" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -4217,5 +4218,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>